<commit_message>
Excel R3.3 con la corrida final de 30 modos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R3.3.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R3.3.xlsx
@@ -13972,10 +13972,10 @@
         </is>
       </c>
       <c r="C73" s="16">
-        <v>2.162</v>
+        <v>2.163</v>
       </c>
       <c r="D73" s="16">
-        <v>1.74</v>
+        <v>1.741</v>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
@@ -14061,11 +14061,11 @@
       </c>
       <c r="C76" s="50">
         <f>IF($C$73&gt;0,MAX(1,$C$74/$C$73),1)</f>
-        <v>1.4709522928505352</v>
+        <v>1.4702722409352091</v>
       </c>
       <c r="D76" s="50">
         <f>IF($D$73&gt;0,MAX(1,$D$74/$D$73),1)</f>
-        <v>1.8277004926108373</v>
+        <v>1.8266506933617788</v>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
@@ -14119,11 +14119,11 @@
       </c>
       <c r="C78" s="21">
         <f>$C$76</f>
-        <v>1.4709522928505352</v>
+        <v>1.4702722409352091</v>
       </c>
       <c r="D78" s="21">
         <f>$D$76</f>
-        <v>1.8277004926108373</v>
+        <v>1.8266506933617788</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14179,11 +14179,11 @@
       </c>
       <c r="C80" s="21">
         <f>IF($C$73&gt;0,MAX(1,$C$79/$C$73),1)</f>
-        <v>1.4709522928505352</v>
+        <v>1.4702722409352091</v>
       </c>
       <c r="D80" s="21">
         <f>IF($D$73&gt;0,MAX(1,$D$79/$D$73),1)</f>
-        <v>1.8277004926108373</v>
+        <v>1.8266506933617788</v>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="C92" s="13">
         <f>$C$73</f>
-        <v>2.162</v>
+        <v>2.163</v>
       </c>
       <c r="D92" s="53">
         <v>1.82038061</v>
@@ -14483,7 +14483,7 @@
       </c>
       <c r="C93" s="21">
         <f>$C$76</f>
-        <v>1.4709522928505352</v>
+        <v>1.4702722409352091</v>
       </c>
       <c r="D93" s="21">
         <f>MAX(1,D91/D92)</f>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="C101" s="13">
         <f>$D$73</f>
-        <v>1.74</v>
+        <v>1.741</v>
       </c>
       <c r="D101" s="53">
         <v>2.72429032</v>
@@ -14731,7 +14731,7 @@
       </c>
       <c r="C102" s="21">
         <f>$D$76</f>
-        <v>1.8277004926108373</v>
+        <v>1.8266506933617788</v>
       </c>
       <c r="D102" s="21">
         <f>MAX(1,D100/D101)</f>
@@ -14793,11 +14793,11 @@
       </c>
       <c r="C104" s="13">
         <f>$C$76</f>
-        <v>1.4709522928505352</v>
+        <v>1.4702722409352091</v>
       </c>
       <c r="D104" s="13">
         <f>$D$76</f>
-        <v>1.8277004926108373</v>
+        <v>1.8266506933617788</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14823,11 +14823,11 @@
       </c>
       <c r="C105" s="13">
         <f>-$C$76</f>
-        <v>-1.4709522928505352</v>
+        <v>-1.4702722409352091</v>
       </c>
       <c r="D105" s="13">
         <f>-$D$76</f>
-        <v>-1.8277004926108373</v>
+        <v>-1.8266506933617788</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14853,11 +14853,11 @@
       </c>
       <c r="C106" s="55">
         <f>DATOS!$C$26/$C$12*$C$76</f>
-        <v>0.30259590024353866</v>
+        <v>0.30245600384952875</v>
       </c>
       <c r="D106" s="55">
         <f>DATOS!$C$26/$D$12*$D$76</f>
-        <v>0.37598410133708654</v>
+        <v>0.37576814263442304</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Excel R3.3 con la corrida final de 25 modos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R3.3.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R3.3.xlsx
@@ -13972,10 +13972,10 @@
         </is>
       </c>
       <c r="C73" s="16">
-        <v>2.163</v>
+        <v>2.162</v>
       </c>
       <c r="D73" s="16">
-        <v>1.741</v>
+        <v>1.74</v>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
@@ -14061,11 +14061,11 @@
       </c>
       <c r="C76" s="50">
         <f>IF($C$73&gt;0,MAX(1,$C$74/$C$73),1)</f>
-        <v>1.4702722409352091</v>
+        <v>1.4709522928505352</v>
       </c>
       <c r="D76" s="50">
         <f>IF($D$73&gt;0,MAX(1,$D$74/$D$73),1)</f>
-        <v>1.8266506933617788</v>
+        <v>1.8277004926108373</v>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
@@ -14119,11 +14119,11 @@
       </c>
       <c r="C78" s="21">
         <f>$C$76</f>
-        <v>1.4702722409352091</v>
+        <v>1.4709522928505352</v>
       </c>
       <c r="D78" s="21">
         <f>$D$76</f>
-        <v>1.8266506933617788</v>
+        <v>1.8277004926108373</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14179,11 +14179,11 @@
       </c>
       <c r="C80" s="21">
         <f>IF($C$73&gt;0,MAX(1,$C$79/$C$73),1)</f>
-        <v>1.4702722409352091</v>
+        <v>1.4709522928505352</v>
       </c>
       <c r="D80" s="21">
         <f>IF($D$73&gt;0,MAX(1,$D$79/$D$73),1)</f>
-        <v>1.8266506933617788</v>
+        <v>1.8277004926108373</v>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="C92" s="13">
         <f>$C$73</f>
-        <v>2.163</v>
+        <v>2.162</v>
       </c>
       <c r="D92" s="53">
         <v>1.82038061</v>
@@ -14483,7 +14483,7 @@
       </c>
       <c r="C93" s="21">
         <f>$C$76</f>
-        <v>1.4702722409352091</v>
+        <v>1.4709522928505352</v>
       </c>
       <c r="D93" s="21">
         <f>MAX(1,D91/D92)</f>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="C101" s="13">
         <f>$D$73</f>
-        <v>1.741</v>
+        <v>1.74</v>
       </c>
       <c r="D101" s="53">
         <v>2.72429032</v>
@@ -14731,7 +14731,7 @@
       </c>
       <c r="C102" s="21">
         <f>$D$76</f>
-        <v>1.8266506933617788</v>
+        <v>1.8277004926108373</v>
       </c>
       <c r="D102" s="21">
         <f>MAX(1,D100/D101)</f>
@@ -14793,11 +14793,11 @@
       </c>
       <c r="C104" s="13">
         <f>$C$76</f>
-        <v>1.4702722409352091</v>
+        <v>1.4709522928505352</v>
       </c>
       <c r="D104" s="13">
         <f>$D$76</f>
-        <v>1.8266506933617788</v>
+        <v>1.8277004926108373</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14823,11 +14823,11 @@
       </c>
       <c r="C105" s="13">
         <f>-$C$76</f>
-        <v>-1.4702722409352091</v>
+        <v>-1.4709522928505352</v>
       </c>
       <c r="D105" s="13">
         <f>-$D$76</f>
-        <v>-1.8266506933617788</v>
+        <v>-1.8277004926108373</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14853,11 +14853,11 @@
       </c>
       <c r="C106" s="55">
         <f>DATOS!$C$26/$C$12*$C$76</f>
-        <v>0.30245600384952875</v>
+        <v>0.30259590024353866</v>
       </c>
       <c r="D106" s="55">
         <f>DATOS!$C$26/$D$12*$D$76</f>
-        <v>0.37576814263442304</v>
+        <v>0.37598410133708654</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>

</xml_diff>